<commit_message>
Actualizacion de resultados despues de la corrida de simulaciones
</commit_message>
<xml_diff>
--- a/resultados/Resultados_Cortocircuito.xlsx
+++ b/resultados/Resultados_Cortocircuito.xlsx
@@ -2938,10 +2938,10 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3.68884860943635</v>
+        <v>3.688848609436351</v>
       </c>
       <c r="F3" t="n">
-        <v>28112.80173086462</v>
+        <v>28112.80173086463</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2971,10 +2971,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4.259515472767732</v>
+        <v>3.890953144182498</v>
       </c>
       <c r="F4" t="n">
-        <v>32461.86727456035</v>
+        <v>29653.04512813845</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -3037,10 +3037,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4.510449866195843</v>
+        <v>4.510449866195846</v>
       </c>
       <c r="F6" t="n">
-        <v>34374.2441695767</v>
+        <v>34374.24416957672</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -3070,10 +3070,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>5.208218883339058</v>
+        <v>4.644769057829843</v>
       </c>
       <c r="F7" t="n">
-        <v>39691.95820715137</v>
+        <v>35397.8938778887</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -3136,10 +3136,10 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>5.78349383116875</v>
+        <v>5.783493831168753</v>
       </c>
       <c r="F9" t="n">
-        <v>44076.14207083689</v>
+        <v>44076.14207083692</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -3169,10 +3169,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>6.678203427068497</v>
+        <v>5.742794930900801</v>
       </c>
       <c r="F10" t="n">
-        <v>50894.74487602896</v>
+        <v>43765.97479778311</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -3235,10 +3235,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3.561131837190445</v>
+        <v>3.561131837190446</v>
       </c>
       <c r="F12" t="n">
-        <v>27139.469215491</v>
+        <v>27139.46921549101</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -3268,10 +3268,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4.112040812952518</v>
+        <v>3.770159792089812</v>
       </c>
       <c r="F13" t="n">
-        <v>31337.95943483328</v>
+        <v>28732.47616005952</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -3337,7 +3337,7 @@
         <v>1.32181773992302</v>
       </c>
       <c r="F15" t="n">
-        <v>10073.60398356749</v>
+        <v>10073.6039835675</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -3367,10 +3367,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1.526303655997092</v>
+        <v>1.485660619385841</v>
       </c>
       <c r="F16" t="n">
-        <v>11631.99594376859</v>
+        <v>11322.25440895213</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1.887961229584406</v>
+        <v>1.887961229584407</v>
       </c>
       <c r="F18" t="n">
         <v>14388.19679048192</v>
@@ -3466,10 +3466,10 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2.180029848192149</v>
+        <v>2.092797194481272</v>
       </c>
       <c r="F19" t="n">
-        <v>16614.05857990938</v>
+        <v>15949.25648096778</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -3532,10 +3532,10 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3.369621763477802</v>
+        <v>3.369621763477803</v>
       </c>
       <c r="F21" t="n">
-        <v>25679.96645412139</v>
+        <v>25679.9664541214</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -3565,10 +3565,10 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>3.890904062653652</v>
+        <v>3.587140498942058</v>
       </c>
       <c r="F22" t="n">
-        <v>29652.67107665649</v>
+        <v>27337.68183642585</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -3631,10 +3631,10 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1.607299297756171</v>
+        <v>1.607299297756172</v>
       </c>
       <c r="F24" t="n">
-        <v>12249.26562841012</v>
+        <v>12249.26562841013</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -3664,10 +3664,10 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1.85594932707515</v>
+        <v>1.79421313535318</v>
       </c>
       <c r="F25" t="n">
-        <v>14144.23333099801</v>
+        <v>13673.74036659209</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -3730,10 +3730,10 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1.070180344926783</v>
+        <v>1.070180344926784</v>
       </c>
       <c r="F27" t="n">
-        <v>8155.869497119867</v>
+        <v>8155.86949711987</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -3763,10 +3763,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1.235737783271109</v>
+        <v>1.209785709679961</v>
       </c>
       <c r="F28" t="n">
-        <v>9417.586615935172</v>
+        <v>9219.805254697843</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.6670697247609172</v>
+        <v>0.6670697247609173</v>
       </c>
       <c r="F30" t="n">
         <v>5083.754010640072</v>
@@ -3862,10 +3862,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.7702657333933089</v>
+        <v>0.7606483006177469</v>
       </c>
       <c r="F31" t="n">
-        <v>5870.213211670365</v>
+        <v>5796.918531024578</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -3928,10 +3928,10 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.6618948878760713</v>
+        <v>0.6618948878760714</v>
       </c>
       <c r="F33" t="n">
-        <v>5044.316457426017</v>
+        <v>5044.316457426018</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -3961,10 +3961,10 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.76429034646018</v>
+        <v>0.7548277297037239</v>
       </c>
       <c r="F34" t="n">
-        <v>5824.674647770906</v>
+        <v>5752.559823636104</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -4060,10 +4060,10 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.3287168665993284</v>
+        <v>0.3270534792264616</v>
       </c>
       <c r="F37" t="n">
-        <v>2505.158946522889</v>
+        <v>2492.482232359178</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -4126,10 +4126,10 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>7.032977150626407</v>
+        <v>7.032977150626413</v>
       </c>
       <c r="F39" t="n">
-        <v>53598.48374028885</v>
+        <v>53598.4837402889</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -4159,10 +4159,10 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>8.120982475265858</v>
+        <v>6.769751244807761</v>
       </c>
       <c r="F40" t="n">
-        <v>61890.1978256732</v>
+        <v>51592.43294119207</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -4225,10 +4225,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1.740221595690985</v>
+        <v>1.740221595690987</v>
       </c>
       <c r="F42" t="n">
-        <v>34662.75053190178</v>
+        <v>34662.75053190182</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -4258,10 +4258,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2.009434808829138</v>
+        <v>1.779829268760349</v>
       </c>
       <c r="F43" t="n">
-        <v>40025.0966089795</v>
+        <v>35451.6793063475</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -4324,10 +4324,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>5.197884771746993</v>
+        <v>5.197884771746995</v>
       </c>
       <c r="F45" t="n">
-        <v>345115.0198012501</v>
+        <v>345115.0198012502</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -4357,10 +4357,10 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>6.002000341211034</v>
+        <v>2.622105831227587</v>
       </c>
       <c r="F46" t="n">
-        <v>398504.498957558</v>
+        <v>174095.4533628375</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -4423,10 +4423,10 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>3.688848708001731</v>
+        <v>3.688848708001732</v>
       </c>
       <c r="F48" t="n">
-        <v>28112.80248203369</v>
+        <v>28112.8024820337</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -4456,10 +4456,10 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>4.260296460142946</v>
+        <v>3.892715232156609</v>
       </c>
       <c r="F49" t="n">
-        <v>32467.81919765568</v>
+        <v>29666.4740418981</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -4522,7 +4522,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>4.51045007890812</v>
+        <v>4.510450078908121</v>
       </c>
       <c r="F51" t="n">
         <v>34374.24579066195</v>
@@ -4555,10 +4555,10 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>5.209458514554782</v>
+        <v>4.647392882476122</v>
       </c>
       <c r="F52" t="n">
-        <v>39701.4054657073</v>
+        <v>35417.8901070288</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -4621,10 +4621,10 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>5.783494354719819</v>
+        <v>5.783494354719823</v>
       </c>
       <c r="F54" t="n">
-        <v>44076.14606083186</v>
+        <v>44076.14606083189</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -4654,10 +4654,10 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>6.680382630373627</v>
+        <v>5.746980693067954</v>
       </c>
       <c r="F55" t="n">
-        <v>50911.35263550482</v>
+        <v>43797.87458938656</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -4720,10 +4720,10 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>3.561133266835946</v>
+        <v>3.561133266835948</v>
       </c>
       <c r="F57" t="n">
-        <v>27139.48011085288</v>
+        <v>27139.4801108529</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4753,10 +4753,10 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>4.114801663461343</v>
+        <v>3.774327240346848</v>
       </c>
       <c r="F58" t="n">
-        <v>31358.99994128415</v>
+        <v>28764.23638092465</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -4852,10 +4852,10 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1.526381628303356</v>
+        <v>1.48586732189782</v>
       </c>
       <c r="F61" t="n">
-        <v>11632.59017254255</v>
+        <v>11323.82969364169</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>2.180200885643565</v>
+        <v>2.093235783510627</v>
       </c>
       <c r="F64" t="n">
-        <v>16615.36206033628</v>
+        <v>15952.59897824242</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -5017,10 +5017,10 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>3.369621831822944</v>
+        <v>3.369621831822945</v>
       </c>
       <c r="F66" t="n">
-        <v>25679.96697498133</v>
+        <v>25679.96697498134</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -5050,10 +5050,10 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>3.891538539505143</v>
+        <v>3.588607272632167</v>
       </c>
       <c r="F67" t="n">
-        <v>29657.50643961585</v>
+        <v>27348.86015310401</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -5116,10 +5116,10 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1.60729956541263</v>
+        <v>1.607299565412631</v>
       </c>
       <c r="F69" t="n">
-        <v>12249.26766822627</v>
+        <v>12249.26766822628</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -5149,10 +5149,10 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>1.856585799661717</v>
+        <v>1.795229024666307</v>
       </c>
       <c r="F70" t="n">
-        <v>14149.08390350119</v>
+        <v>13681.48248286311</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -5248,10 +5248,10 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>1.236025747703756</v>
+        <v>1.210251089875468</v>
       </c>
       <c r="F73" t="n">
-        <v>9419.781199627174</v>
+        <v>9223.351928077789</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -5314,7 +5314,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.667069768016006</v>
+        <v>0.6670697680160059</v>
       </c>
       <c r="F75" t="n">
         <v>5083.754340288117</v>
@@ -5347,10 +5347,10 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.7703789813431208</v>
+        <v>0.7608326576658677</v>
       </c>
       <c r="F76" t="n">
-        <v>5871.076276950773</v>
+        <v>5798.323520410222</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -5446,10 +5446,10 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.7644018596375778</v>
+        <v>0.7550092772006374</v>
       </c>
       <c r="F79" t="n">
-        <v>5825.524492310077</v>
+        <v>5753.943401366133</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -5545,10 +5545,10 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>0.3287376808193624</v>
+        <v>0.3270875278080067</v>
       </c>
       <c r="F82" t="n">
-        <v>2505.31757218172</v>
+        <v>2492.74171739734</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -5611,10 +5611,10 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>7.032978197800823</v>
+        <v>7.032978197800827</v>
       </c>
       <c r="F84" t="n">
-        <v>53598.49172082962</v>
+        <v>53598.49172082965</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -5644,10 +5644,10 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>8.12429007884397</v>
+        <v>6.7756161410439</v>
       </c>
       <c r="F85" t="n">
-        <v>61915.40515008275</v>
+        <v>51637.12945289951</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -5713,7 +5713,7 @@
         <v>1.740221775703433</v>
       </c>
       <c r="F87" t="n">
-        <v>34662.75411749488</v>
+        <v>34662.75411749489</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -5743,10 +5743,10 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>2.010000853578232</v>
+        <v>1.780933820843935</v>
       </c>
       <c r="F88" t="n">
-        <v>40036.37141902456</v>
+        <v>35473.68042012383</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -5809,10 +5809,10 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>5.197884901325367</v>
+        <v>5.197884901325369</v>
       </c>
       <c r="F90" t="n">
-        <v>345115.0284046426</v>
+        <v>345115.0284046428</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -5842,10 +5842,10 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>6.002378077569922</v>
+        <v>2.623812897302295</v>
       </c>
       <c r="F91" t="n">
-        <v>398529.5788692338</v>
+        <v>174208.7944944795</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -5941,10 +5941,10 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>13.49317951817623</v>
+        <v>13.22010829529497</v>
       </c>
       <c r="F94" t="n">
-        <v>6232.232754501895</v>
+        <v>6106.106557391719</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -7001,10 +7001,10 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>4.259515472198363</v>
+        <v>3.890953143652293</v>
       </c>
       <c r="H27" t="n">
-        <v>4.259515472198363</v>
+        <v>3.890953143652293</v>
       </c>
     </row>
     <row r="28">
@@ -8597,10 +8597,10 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>5.208218882875124</v>
+        <v>4.64476905740404</v>
       </c>
       <c r="H69" t="n">
-        <v>5.208218882875124</v>
+        <v>4.64476905740404</v>
       </c>
     </row>
     <row r="70">
@@ -9927,10 +9927,10 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>6.678203426799785</v>
+        <v>5.742794930654815</v>
       </c>
       <c r="H104" t="n">
-        <v>6.678203426799785</v>
+        <v>5.742794930654815</v>
       </c>
     </row>
     <row r="105">
@@ -11143,10 +11143,10 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>4.112040737848774</v>
+        <v>3.770159723200935</v>
       </c>
       <c r="H136" t="n">
-        <v>4.112040737848774</v>
+        <v>3.770159723200935</v>
       </c>
     </row>
     <row r="137">
@@ -12473,10 +12473,10 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>1.52630365549084</v>
+        <v>1.485660618889213</v>
       </c>
       <c r="H171" t="n">
-        <v>1.52630365549084</v>
+        <v>1.485660618889213</v>
       </c>
     </row>
     <row r="172">
@@ -12853,10 +12853,10 @@
         </is>
       </c>
       <c r="G181" t="n">
-        <v>1.526303655592851</v>
+        <v>1.485660618990435</v>
       </c>
       <c r="H181" t="n">
-        <v>1.526303655592851</v>
+        <v>1.485660618990435</v>
       </c>
     </row>
     <row r="182">
@@ -14069,10 +14069,10 @@
         </is>
       </c>
       <c r="G213" t="n">
-        <v>2.180029847715572</v>
+        <v>2.092797194018331</v>
       </c>
       <c r="H213" t="n">
-        <v>2.180029847715572</v>
+        <v>2.092797194018331</v>
       </c>
     </row>
     <row r="214">
@@ -14183,10 +14183,10 @@
         </is>
       </c>
       <c r="G216" t="n">
-        <v>2.180029847812669</v>
+        <v>2.092797194114259</v>
       </c>
       <c r="H216" t="n">
-        <v>2.180029847812669</v>
+        <v>2.092797194114259</v>
       </c>
     </row>
     <row r="217">
@@ -15399,10 +15399,10 @@
         </is>
       </c>
       <c r="G248" t="n">
-        <v>3.890904062271945</v>
+        <v>3.587140498580838</v>
       </c>
       <c r="H248" t="n">
-        <v>3.890904062271945</v>
+        <v>3.587140498580838</v>
       </c>
     </row>
     <row r="249">
@@ -15475,10 +15475,10 @@
         </is>
       </c>
       <c r="G250" t="n">
-        <v>3.890904062350227</v>
+        <v>3.587140498657663</v>
       </c>
       <c r="H250" t="n">
-        <v>3.890904062350227</v>
+        <v>3.587140498657663</v>
       </c>
     </row>
     <row r="251">
@@ -16615,10 +16615,10 @@
         </is>
       </c>
       <c r="G280" t="n">
-        <v>1.855949250225881</v>
+        <v>1.794213061046247</v>
       </c>
       <c r="H280" t="n">
-        <v>1.855949250225881</v>
+        <v>1.794213061046247</v>
       </c>
     </row>
     <row r="281">
@@ -16691,10 +16691,10 @@
         </is>
       </c>
       <c r="G282" t="n">
-        <v>1.855949250357805</v>
+        <v>1.794213061176111</v>
       </c>
       <c r="H282" t="n">
-        <v>1.855949250357805</v>
+        <v>1.794213061176111</v>
       </c>
     </row>
     <row r="283">
@@ -17983,10 +17983,10 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>1.235737706908008</v>
+        <v>1.20978563491116</v>
       </c>
       <c r="H316" t="n">
-        <v>1.235737706908008</v>
+        <v>1.20978563491116</v>
       </c>
     </row>
     <row r="317">
@@ -18021,10 +18021,10 @@
         </is>
       </c>
       <c r="G317" t="n">
-        <v>1.235737707256873</v>
+        <v>1.20978563525584</v>
       </c>
       <c r="H317" t="n">
-        <v>1.235737707256873</v>
+        <v>1.20978563525584</v>
       </c>
     </row>
     <row r="318">
@@ -18059,10 +18059,10 @@
         </is>
       </c>
       <c r="G318" t="n">
-        <v>1.235737706995846</v>
+        <v>1.209785634998724</v>
       </c>
       <c r="H318" t="n">
-        <v>1.235737706995846</v>
+        <v>1.209785634998724</v>
       </c>
     </row>
     <row r="319">
@@ -19351,10 +19351,10 @@
         </is>
       </c>
       <c r="G352" t="n">
-        <v>0.7702656577782832</v>
+        <v>0.7606482259409153</v>
       </c>
       <c r="H352" t="n">
-        <v>0.7702656577782832</v>
+        <v>0.7606482259409153</v>
       </c>
     </row>
     <row r="353">
@@ -19389,10 +19389,10 @@
         </is>
       </c>
       <c r="G353" t="n">
-        <v>0.7702656579957394</v>
+        <v>0.7606482261576315</v>
       </c>
       <c r="H353" t="n">
-        <v>0.7702656579957394</v>
+        <v>0.7606482261576315</v>
       </c>
     </row>
     <row r="354">
@@ -19427,10 +19427,10 @@
         </is>
       </c>
       <c r="G354" t="n">
-        <v>0.770265657833035</v>
+        <v>0.7606482259959709</v>
       </c>
       <c r="H354" t="n">
-        <v>0.770265657833035</v>
+        <v>0.7606482259959709</v>
       </c>
     </row>
     <row r="355">
@@ -19465,10 +19465,10 @@
         </is>
       </c>
       <c r="G355" t="n">
-        <v>0.7702656582541295</v>
+        <v>0.7606482264137829</v>
       </c>
       <c r="H355" t="n">
-        <v>0.7702656582541295</v>
+        <v>0.7606482264137829</v>
       </c>
     </row>
     <row r="356">
@@ -20643,10 +20643,10 @@
         </is>
       </c>
       <c r="G386" t="n">
-        <v>0.7642902717583919</v>
+        <v>0.7548276559248689</v>
       </c>
       <c r="H386" t="n">
-        <v>0.7642902717583919</v>
+        <v>0.7548276559248689</v>
       </c>
     </row>
     <row r="387">
@@ -20719,10 +20719,10 @@
         </is>
       </c>
       <c r="G388" t="n">
-        <v>0.7642902708594427</v>
+        <v>0.7548276550331143</v>
       </c>
       <c r="H388" t="n">
-        <v>0.7642902708594427</v>
+        <v>0.7548276550331143</v>
       </c>
     </row>
     <row r="389">
@@ -20757,10 +20757,10 @@
         </is>
       </c>
       <c r="G389" t="n">
-        <v>0.7642902710752122</v>
+        <v>0.7548276552481716</v>
       </c>
       <c r="H389" t="n">
-        <v>0.7642902710752122</v>
+        <v>0.7548276552481716</v>
       </c>
     </row>
     <row r="390">
@@ -20795,10 +20795,10 @@
         </is>
       </c>
       <c r="G390" t="n">
-        <v>0.7642902709137697</v>
+        <v>0.7548276550877484</v>
       </c>
       <c r="H390" t="n">
-        <v>0.7642902709137697</v>
+        <v>0.7548276550877484</v>
       </c>
     </row>
     <row r="391">
@@ -20833,10 +20833,10 @@
         </is>
       </c>
       <c r="G391" t="n">
-        <v>0.7642902713315979</v>
+        <v>0.7548276555023631</v>
       </c>
       <c r="H391" t="n">
-        <v>0.7642902713315979</v>
+        <v>0.7548276555023631</v>
       </c>
     </row>
     <row r="392">
@@ -22011,10 +22011,10 @@
         </is>
       </c>
       <c r="G422" t="n">
-        <v>0.3287168134875439</v>
+        <v>0.3270534263825842</v>
       </c>
       <c r="H422" t="n">
-        <v>0.3287168134875439</v>
+        <v>0.3270534263825842</v>
       </c>
     </row>
     <row r="423">
@@ -22087,10 +22087,10 @@
         </is>
       </c>
       <c r="G424" t="n">
-        <v>0.3287168131009114</v>
+        <v>0.3270534259962124</v>
       </c>
       <c r="H424" t="n">
-        <v>0.3287168131009114</v>
+        <v>0.3270534259962124</v>
       </c>
     </row>
     <row r="425">
@@ -22125,10 +22125,10 @@
         </is>
       </c>
       <c r="G425" t="n">
-        <v>0.3287168131937127</v>
+        <v>0.327053426089393</v>
       </c>
       <c r="H425" t="n">
-        <v>0.3287168131937127</v>
+        <v>0.327053426089393</v>
       </c>
     </row>
     <row r="426">
@@ -22163,10 +22163,10 @@
         </is>
       </c>
       <c r="G426" t="n">
-        <v>0.3287168131242773</v>
+        <v>0.3270534260198846</v>
       </c>
       <c r="H426" t="n">
-        <v>0.3287168131242773</v>
+        <v>0.3270534260198846</v>
       </c>
     </row>
     <row r="427">
@@ -22201,10 +22201,10 @@
         </is>
       </c>
       <c r="G427" t="n">
-        <v>0.3287168133039824</v>
+        <v>0.3270534261995297</v>
       </c>
       <c r="H427" t="n">
-        <v>0.3287168133039824</v>
+        <v>0.3270534261995297</v>
       </c>
     </row>
     <row r="428">
@@ -22353,10 +22353,10 @@
         </is>
       </c>
       <c r="G431" t="n">
-        <v>0.3287168295519504</v>
+        <v>0.3270534423661279</v>
       </c>
       <c r="H431" t="n">
-        <v>0.3287168295519504</v>
+        <v>0.3270534423661279</v>
       </c>
     </row>
     <row r="432">
@@ -27521,10 +27521,10 @@
         </is>
       </c>
       <c r="G567" t="n">
-        <v>4.260296459573478</v>
+        <v>3.892715231626212</v>
       </c>
       <c r="H567" t="n">
-        <v>4.260296459573478</v>
+        <v>3.892715231626212</v>
       </c>
     </row>
     <row r="568">
@@ -27559,10 +27559,10 @@
         </is>
       </c>
       <c r="G568" t="n">
-        <v>0.001734669245094053</v>
+        <v>0.002532689533522798</v>
       </c>
       <c r="H568" t="n">
-        <v>0.001734669245094053</v>
+        <v>0.002532689533522798</v>
       </c>
     </row>
     <row r="569">
@@ -28471,10 +28471,10 @@
         </is>
       </c>
       <c r="G592" t="n">
-        <v>1.152119218139538e-06</v>
+        <v>1.152119218142447e-06</v>
       </c>
       <c r="H592" t="n">
-        <v>1.152119218139538e-06</v>
+        <v>1.152119218142447e-06</v>
       </c>
     </row>
     <row r="593">
@@ -28927,10 +28927,10 @@
         </is>
       </c>
       <c r="G604" t="n">
-        <v>0.00212114052478035</v>
+        <v>0.003023700067991046</v>
       </c>
       <c r="H604" t="n">
-        <v>0.00212114052478035</v>
+        <v>0.003023700067991046</v>
       </c>
     </row>
     <row r="605">
@@ -29117,10 +29117,10 @@
         </is>
       </c>
       <c r="G609" t="n">
-        <v>5.209458514090746</v>
+        <v>4.647392882050136</v>
       </c>
       <c r="H609" t="n">
-        <v>5.209458514090746</v>
+        <v>4.647392882050136</v>
       </c>
     </row>
     <row r="610">
@@ -29839,10 +29839,10 @@
         </is>
       </c>
       <c r="G628" t="n">
-        <v>1.477297138383368e-06</v>
+        <v>1.477297138384891e-06</v>
       </c>
       <c r="H628" t="n">
-        <v>1.477297138383368e-06</v>
+        <v>1.477297138384891e-06</v>
       </c>
     </row>
     <row r="629">
@@ -30295,10 +30295,10 @@
         </is>
       </c>
       <c r="G640" t="n">
-        <v>0.002720058194036939</v>
+        <v>0.003739117038874551</v>
       </c>
       <c r="H640" t="n">
-        <v>0.002720058194036939</v>
+        <v>0.003739117038874551</v>
       </c>
     </row>
     <row r="641">
@@ -30447,10 +30447,10 @@
         </is>
       </c>
       <c r="G644" t="n">
-        <v>6.680382630104837</v>
+        <v>5.746980692821861</v>
       </c>
       <c r="H644" t="n">
-        <v>6.680382630104837</v>
+        <v>5.746980692821861</v>
       </c>
     </row>
     <row r="645">
@@ -31207,10 +31207,10 @@
         </is>
       </c>
       <c r="G664" t="n">
-        <v>1.796457423801748e-06</v>
+        <v>1.796457423802511e-06</v>
       </c>
       <c r="H664" t="n">
-        <v>1.796457423801748e-06</v>
+        <v>1.796457423802511e-06</v>
       </c>
     </row>
     <row r="665">
@@ -31663,10 +31663,10 @@
         </is>
       </c>
       <c r="G676" t="n">
-        <v>4.112040737848764</v>
+        <v>3.770878936626446</v>
       </c>
       <c r="H676" t="n">
-        <v>4.112040737848764</v>
+        <v>3.770878936626446</v>
       </c>
     </row>
     <row r="677">
@@ -32993,10 +32993,10 @@
         </is>
       </c>
       <c r="G711" t="n">
-        <v>1.52638162779708</v>
+        <v>1.485867321401141</v>
       </c>
       <c r="H711" t="n">
-        <v>1.52638162779708</v>
+        <v>1.485867321401141</v>
       </c>
     </row>
     <row r="712">
@@ -33031,10 +33031,10 @@
         </is>
       </c>
       <c r="G712" t="n">
-        <v>0.0006214983607694887</v>
+        <v>0.0009667392524747419</v>
       </c>
       <c r="H712" t="n">
-        <v>0.0006214983607694887</v>
+        <v>0.0009667392524747419</v>
       </c>
     </row>
     <row r="713">
@@ -33373,10 +33373,10 @@
         </is>
       </c>
       <c r="G721" t="n">
-        <v>1.526381627899095</v>
+        <v>1.485867321502368</v>
       </c>
       <c r="H721" t="n">
-        <v>1.526381627899095</v>
+        <v>1.485867321502368</v>
       </c>
     </row>
     <row r="722">
@@ -34399,10 +34399,10 @@
         </is>
       </c>
       <c r="G748" t="n">
-        <v>0.0008877146131766779</v>
+        <v>0.001361907060617385</v>
       </c>
       <c r="H748" t="n">
-        <v>0.0008877146131766779</v>
+        <v>0.001361907060617385</v>
       </c>
     </row>
     <row r="749">
@@ -34589,10 +34589,10 @@
         </is>
       </c>
       <c r="G753" t="n">
-        <v>2.180200885166955</v>
+        <v>2.093235783047616</v>
       </c>
       <c r="H753" t="n">
-        <v>2.180200885166955</v>
+        <v>2.093235783047616</v>
       </c>
     </row>
     <row r="754">
@@ -34703,10 +34703,10 @@
         </is>
       </c>
       <c r="G756" t="n">
-        <v>2.180200885264057</v>
+        <v>2.09323578314355</v>
       </c>
       <c r="H756" t="n">
-        <v>2.180200885264057</v>
+        <v>2.09323578314355</v>
       </c>
     </row>
     <row r="757">
@@ -35767,10 +35767,10 @@
         </is>
       </c>
       <c r="G784" t="n">
-        <v>0.001584521707344312</v>
+        <v>0.002334829941981689</v>
       </c>
       <c r="H784" t="n">
-        <v>0.001584521707344312</v>
+        <v>0.002334829941981689</v>
       </c>
     </row>
     <row r="785">
@@ -35919,10 +35919,10 @@
         </is>
       </c>
       <c r="G788" t="n">
-        <v>3.891538539123382</v>
+        <v>3.588607272270846</v>
       </c>
       <c r="H788" t="n">
-        <v>3.891538539123382</v>
+        <v>3.588607272270846</v>
       </c>
     </row>
     <row r="789">
@@ -35995,10 +35995,10 @@
         </is>
       </c>
       <c r="G790" t="n">
-        <v>3.89153853920167</v>
+        <v>3.588607272347679</v>
       </c>
       <c r="H790" t="n">
-        <v>3.89153853920167</v>
+        <v>3.588607272347679</v>
       </c>
     </row>
     <row r="791">
@@ -37135,10 +37135,10 @@
         </is>
       </c>
       <c r="G820" t="n">
-        <v>1.855340035593219</v>
+        <v>1.793588824620628</v>
       </c>
       <c r="H820" t="n">
-        <v>1.855340035593219</v>
+        <v>1.793588824620628</v>
       </c>
     </row>
     <row r="821">
@@ -37211,10 +37211,10 @@
         </is>
       </c>
       <c r="G822" t="n">
-        <v>1.856585722918973</v>
+        <v>1.79522895044849</v>
       </c>
       <c r="H822" t="n">
-        <v>1.856585722918973</v>
+        <v>1.79522895044849</v>
       </c>
     </row>
     <row r="823">
@@ -38503,10 +38503,10 @@
         </is>
       </c>
       <c r="G856" t="n">
-        <v>1.235196352560209</v>
+        <v>1.209145326679041</v>
       </c>
       <c r="H856" t="n">
-        <v>1.235196352560209</v>
+        <v>1.209145326679041</v>
       </c>
     </row>
     <row r="857">
@@ -38541,10 +38541,10 @@
         </is>
       </c>
       <c r="G857" t="n">
-        <v>1.236025671672294</v>
+        <v>1.210251015423395</v>
       </c>
       <c r="H857" t="n">
-        <v>1.236025671672294</v>
+        <v>1.210251015423395</v>
       </c>
     </row>
     <row r="858">
@@ -38579,10 +38579,10 @@
         </is>
       </c>
       <c r="G858" t="n">
-        <v>1.236025671411323</v>
+        <v>1.210251015166346</v>
       </c>
       <c r="H858" t="n">
-        <v>1.236025671411323</v>
+        <v>1.210251015166346</v>
       </c>
     </row>
     <row r="859">
@@ -39871,10 +39871,10 @@
         </is>
       </c>
       <c r="G892" t="n">
-        <v>0.769862015400936</v>
+        <v>0.7601374843705906</v>
       </c>
       <c r="H892" t="n">
-        <v>0.769862015400936</v>
+        <v>0.7601374843705906</v>
       </c>
     </row>
     <row r="893">
@@ -39909,10 +39909,10 @@
         </is>
       </c>
       <c r="G893" t="n">
-        <v>0.77037890593477</v>
+        <v>0.7608325831881317</v>
       </c>
       <c r="H893" t="n">
-        <v>0.77037890593477</v>
+        <v>0.7608325831881317</v>
       </c>
     </row>
     <row r="894">
@@ -39947,10 +39947,10 @@
         </is>
       </c>
       <c r="G894" t="n">
-        <v>0.7703789057721149</v>
+        <v>0.7608325830265367</v>
       </c>
       <c r="H894" t="n">
-        <v>0.7703789057721149</v>
+        <v>0.7608325830265367</v>
       </c>
     </row>
     <row r="895">
@@ -39985,10 +39985,10 @@
         </is>
       </c>
       <c r="G895" t="n">
-        <v>0.770378906193125</v>
+        <v>0.7608325834442413</v>
       </c>
       <c r="H895" t="n">
-        <v>0.770378906193125</v>
+        <v>0.7608325834442413</v>
       </c>
     </row>
     <row r="896">
@@ -41163,10 +41163,10 @@
         </is>
       </c>
       <c r="G926" t="n">
-        <v>0.7644017849250444</v>
+        <v>0.7550092034042585</v>
       </c>
       <c r="H926" t="n">
-        <v>0.7644017849250444</v>
+        <v>0.7550092034042585</v>
       </c>
     </row>
     <row r="927">
@@ -41239,10 +41239,10 @@
         </is>
       </c>
       <c r="G928" t="n">
-        <v>0.763888904094857</v>
+        <v>0.7543194241666089</v>
       </c>
       <c r="H928" t="n">
-        <v>0.763888904094857</v>
+        <v>0.7543194241666089</v>
       </c>
     </row>
     <row r="929">
@@ -41277,10 +41277,10 @@
         </is>
       </c>
       <c r="G929" t="n">
-        <v>0.7644017842419127</v>
+        <v>0.7550092027276011</v>
       </c>
       <c r="H929" t="n">
-        <v>0.7644017842419127</v>
+        <v>0.7550092027276011</v>
       </c>
     </row>
     <row r="930">
@@ -41315,10 +41315,10 @@
         </is>
       </c>
       <c r="G930" t="n">
-        <v>0.7644017840805194</v>
+        <v>0.755009202567242</v>
       </c>
       <c r="H930" t="n">
-        <v>0.7644017840805194</v>
+        <v>0.755009202567242</v>
       </c>
     </row>
     <row r="931">
@@ -41353,10 +41353,10 @@
         </is>
       </c>
       <c r="G931" t="n">
-        <v>0.7644017844982629</v>
+        <v>0.7550092029817498</v>
       </c>
       <c r="H931" t="n">
-        <v>0.7644017844982629</v>
+        <v>0.7550092029817498</v>
       </c>
     </row>
     <row r="932">
@@ -42531,10 +42531,10 @@
         </is>
       </c>
       <c r="G962" t="n">
-        <v>0.3287376277042838</v>
+        <v>0.3270874749587185</v>
       </c>
       <c r="H962" t="n">
-        <v>0.3287376277042838</v>
+        <v>0.3270874749587185</v>
       </c>
     </row>
     <row r="963">
@@ -42607,10 +42607,10 @@
         </is>
       </c>
       <c r="G964" t="n">
-        <v>0.3285170588364408</v>
+        <v>0.3267886465994193</v>
       </c>
       <c r="H964" t="n">
-        <v>0.3285170588364408</v>
+        <v>0.3267886465994193</v>
       </c>
     </row>
     <row r="965">
@@ -42645,10 +42645,10 @@
         </is>
       </c>
       <c r="G965" t="n">
-        <v>0.3287376274104949</v>
+        <v>0.3270874746655896</v>
       </c>
       <c r="H965" t="n">
-        <v>0.3287376274104949</v>
+        <v>0.3270874746655896</v>
       </c>
     </row>
     <row r="966">
@@ -42683,10 +42683,10 @@
         </is>
       </c>
       <c r="G966" t="n">
-        <v>0.3287376273410864</v>
+        <v>0.3270874745961184</v>
       </c>
       <c r="H966" t="n">
-        <v>0.3287376273410864</v>
+        <v>0.3270874745961184</v>
       </c>
     </row>
     <row r="967">
@@ -42721,10 +42721,10 @@
         </is>
       </c>
       <c r="G967" t="n">
-        <v>0.3287376275207405</v>
+        <v>0.3270874747756929</v>
       </c>
       <c r="H967" t="n">
-        <v>0.3287376275207405</v>
+        <v>0.3270874747756929</v>
       </c>
     </row>
     <row r="968">
@@ -42873,10 +42873,10 @@
         </is>
       </c>
       <c r="G971" t="n">
-        <v>0.3287376437696724</v>
+        <v>0.3270874909438827</v>
       </c>
       <c r="H971" t="n">
-        <v>0.3287376437696724</v>
+        <v>0.3270874909438827</v>
       </c>
     </row>
     <row r="972">
@@ -43519,10 +43519,10 @@
         </is>
       </c>
       <c r="G988" t="n">
-        <v>1.796456939189949e-06</v>
+        <v>1.796456939191196e-06</v>
       </c>
       <c r="H988" t="n">
-        <v>1.796456939189949e-06</v>
+        <v>1.796456939191196e-06</v>
       </c>
     </row>
     <row r="989">
@@ -43975,10 +43975,10 @@
         </is>
       </c>
       <c r="G1000" t="n">
-        <v>0.003307975459374832</v>
+        <v>0.004408370780390941</v>
       </c>
       <c r="H1000" t="n">
-        <v>0.003307975459374832</v>
+        <v>0.004408370780390941</v>
       </c>
     </row>
     <row r="1001">
@@ -44887,10 +44887,10 @@
         </is>
       </c>
       <c r="G1024" t="n">
-        <v>1.201574797885387e-06</v>
+        <v>1.201574797885223e-06</v>
       </c>
       <c r="H1024" t="n">
-        <v>1.201574797885387e-06</v>
+        <v>1.201574797885223e-06</v>
       </c>
     </row>
     <row r="1025">
@@ -45343,10 +45343,10 @@
         </is>
       </c>
       <c r="G1036" t="n">
-        <v>0.002212288545661817</v>
+        <v>0.003093256280283703</v>
       </c>
       <c r="H1036" t="n">
-        <v>0.002212288545661817</v>
+        <v>0.003093256280283703</v>
       </c>
     </row>
     <row r="1037">
@@ -46255,10 +46255,10 @@
         </is>
       </c>
       <c r="G1060" t="n">
-        <v>1.796456701579947e-06</v>
+        <v>1.796456701580907e-06</v>
       </c>
       <c r="H1060" t="n">
-        <v>1.796456701579947e-06</v>
+        <v>1.796456701580907e-06</v>
       </c>
     </row>
     <row r="1061">
@@ -46711,10 +46711,10 @@
         </is>
       </c>
       <c r="G1072" t="n">
-        <v>0.003306836783787871</v>
+        <v>0.007028752804884287</v>
       </c>
       <c r="H1072" t="n">
-        <v>0.003306836783787871</v>
+        <v>0.007028752804884287</v>
       </c>
     </row>
     <row r="1073">
@@ -47623,10 +47623,10 @@
         </is>
       </c>
       <c r="G1096" t="n">
-        <v>1.627507187111494e-06</v>
+        <v>1.627507187111393e-06</v>
       </c>
       <c r="H1096" t="n">
-        <v>1.627507187111494e-06</v>
+        <v>1.627507187111393e-06</v>
       </c>
     </row>
     <row r="1097">
@@ -48079,10 +48079,10 @@
         </is>
       </c>
       <c r="G1108" t="n">
-        <v>0.8148820236966099</v>
+        <v>0.7981979245877346</v>
       </c>
       <c r="H1108" t="n">
-        <v>0.8148820236966099</v>
+        <v>0.7981979245877346</v>
       </c>
     </row>
     <row r="1109">
@@ -48535,7 +48535,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1.4575584590384e-05</v>
+        <v>1.457558459038156e-05</v>
       </c>
     </row>
     <row r="4">
@@ -48560,10 +48560,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.001734641435104472</v>
+        <v>0.002532664968247274</v>
       </c>
       <c r="F4" t="n">
-        <v>9.722064736480907e-06</v>
+        <v>8.883870173392314e-06</v>
       </c>
     </row>
     <row r="5">
@@ -48616,10 +48616,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1.080117711388379e-06</v>
+        <v>1.080117711391294e-06</v>
       </c>
       <c r="F6" t="n">
-        <v>1.78219417148111e-05</v>
+        <v>1.782194171482009e-05</v>
       </c>
     </row>
     <row r="7">
@@ -48644,10 +48644,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.002121106518935765</v>
+        <v>0.003023670740264382</v>
       </c>
       <c r="F7" t="n">
-        <v>1.188806774441816e-05</v>
+        <v>1.060617911975473e-05</v>
       </c>
     </row>
     <row r="8">
@@ -48700,10 +48700,10 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1.384973689378131e-06</v>
+        <v>1.384973689380292e-06</v>
       </c>
       <c r="F9" t="n">
-        <v>2.28520652040357e-05</v>
+        <v>2.285206520403999e-05</v>
       </c>
     </row>
     <row r="10">
@@ -48728,10 +48728,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.002720014586424606</v>
+        <v>0.003739080772117594</v>
       </c>
       <c r="F10" t="n">
-        <v>1.524474012814558e-05</v>
+        <v>1.311563454360099e-05</v>
       </c>
     </row>
     <row r="11">
@@ -48784,10 +48784,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1.684188103667196e-06</v>
+        <v>1.684188103668203e-06</v>
       </c>
       <c r="F12" t="n">
-        <v>2.778910289636059e-05</v>
+        <v>2.778910289635704e-05</v>
       </c>
     </row>
     <row r="13">
@@ -48812,10 +48812,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.003308795782224997</v>
+        <v>0.003872373856521808</v>
       </c>
       <c r="F13" t="n">
-        <v>1.854465489773609e-05</v>
+        <v>1.701043429582167e-05</v>
       </c>
     </row>
     <row r="14">
@@ -48871,7 +48871,7 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>5.222839905531759e-06</v>
+        <v>5.222839905534172e-06</v>
       </c>
     </row>
     <row r="16">
@@ -48896,10 +48896,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.0006214883969892295</v>
+        <v>0.0009667298757952165</v>
       </c>
       <c r="F16" t="n">
-        <v>3.483227315340332e-06</v>
+        <v>3.391014136846287e-06</v>
       </c>
     </row>
     <row r="17">
@@ -48955,7 +48955,7 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>7.459817630502738e-06</v>
+        <v>7.459817630501486e-06</v>
       </c>
     </row>
     <row r="19">
@@ -48980,10 +48980,10 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.0008877003814520619</v>
+        <v>0.001361893851092647</v>
       </c>
       <c r="F19" t="n">
-        <v>4.975253330066328e-06</v>
+        <v>4.777137251155341e-06</v>
       </c>
     </row>
     <row r="20">
@@ -49039,7 +49039,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>1.331423756754693e-05</v>
+        <v>1.331423756754915e-05</v>
       </c>
     </row>
     <row r="22">
@@ -49064,10 +49064,10 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.001584496304500138</v>
+        <v>0.002334807295801106</v>
       </c>
       <c r="F22" t="n">
-        <v>8.880553257668425e-06</v>
+        <v>8.189841590673248e-06</v>
       </c>
     </row>
     <row r="23">
@@ -49123,7 +49123,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>1.254247078750309e-05</v>
+        <v>1.254247078750277e-05</v>
       </c>
     </row>
     <row r="25">
@@ -49148,10 +49148,10 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.001492918434776648</v>
+        <v>0.001841864124097392</v>
       </c>
       <c r="F25" t="n">
-        <v>8.36729043742767e-06</v>
+        <v>8.090878546376809e-06</v>
       </c>
     </row>
     <row r="26">
@@ -49207,7 +49207,7 @@
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>8.351091876435205e-06</v>
+        <v>8.351091876439667e-06</v>
       </c>
     </row>
     <row r="28">
@@ -49232,10 +49232,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.0009939134641618792</v>
+        <v>0.001241690075095034</v>
       </c>
       <c r="F28" t="n">
-        <v>5.570540181653346e-06</v>
+        <v>5.4544539205327e-06</v>
       </c>
     </row>
     <row r="29">
@@ -49291,7 +49291,7 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>5.205440138993542e-06</v>
+        <v>5.205440138994683e-06</v>
       </c>
     </row>
     <row r="31">
@@ -49316,10 +49316,10 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.0006194774202316725</v>
+        <v>0.0007805969910524575</v>
       </c>
       <c r="F31" t="n">
-        <v>3.471955674279752e-06</v>
+        <v>3.428979539618772e-06</v>
       </c>
     </row>
     <row r="32">
@@ -49375,7 +49375,7 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>5.165058583466282e-06</v>
+        <v>5.16505858346641e-06</v>
       </c>
     </row>
     <row r="34">
@@ -49400,10 +49400,10 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.000614671094995783</v>
+        <v>0.0007746223352212203</v>
       </c>
       <c r="F34" t="n">
-        <v>3.445017883658537e-06</v>
+        <v>3.402734269644529e-06</v>
       </c>
     </row>
     <row r="35">
@@ -49459,7 +49459,7 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>2.221461418875165e-06</v>
+        <v>2.22146141887464e-06</v>
       </c>
     </row>
     <row r="37">
@@ -49484,10 +49484,10 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.0002643446604915689</v>
+        <v>0.0003355843590960012</v>
       </c>
       <c r="F37" t="n">
-        <v>1.481559680152781e-06</v>
+        <v>1.474143116585189e-06</v>
       </c>
     </row>
     <row r="38">
@@ -49540,10 +49540,10 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1.684187649346567e-06</v>
+        <v>1.684187649347534e-06</v>
       </c>
       <c r="F39" t="n">
-        <v>2.778909539866034e-05</v>
+        <v>2.778909539866743e-05</v>
       </c>
     </row>
     <row r="40">
@@ -49568,10 +49568,10 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.003307922426354404</v>
+        <v>0.004408328022356672</v>
       </c>
       <c r="F40" t="n">
-        <v>1.85397600422299e-05</v>
+        <v>1.5463164025758e-05</v>
       </c>
     </row>
     <row r="41">
@@ -49624,10 +49624,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1.126482572567595e-06</v>
+        <v>1.126482572566977e-06</v>
       </c>
       <c r="F42" t="n">
-        <v>1.8586961901862e-05</v>
+        <v>1.858696190186552e-05</v>
       </c>
     </row>
     <row r="43">
@@ -49652,10 +49652,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.002212253078548443</v>
+        <v>0.003093225884470105</v>
       </c>
       <c r="F43" t="n">
-        <v>1.239891265420837e-05</v>
+        <v>1.098664294788881e-05</v>
       </c>
     </row>
     <row r="44">
@@ -49708,10 +49708,10 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1.684187426586533e-06</v>
+        <v>1.684187426586979e-06</v>
       </c>
       <c r="F45" t="n">
-        <v>2.778909172310502e-05</v>
+        <v>2.778909172310147e-05</v>
       </c>
     </row>
     <row r="46">
@@ -49736,10 +49736,10 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.003306783769023615</v>
+        <v>0.007028729633609435</v>
       </c>
       <c r="F46" t="n">
-        <v>1.853337826320461e-05</v>
+        <v>8.104911585161725e-06</v>
       </c>
     </row>
     <row r="47">
@@ -49792,10 +49792,10 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1.607635864332865e-06</v>
+        <v>1.607635864332768e-06</v>
       </c>
       <c r="F48" t="n">
-        <v>2.652599098562918e-05</v>
+        <v>2.652599098563603e-05</v>
       </c>
     </row>
     <row r="49">
@@ -49820,10 +49820,10 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.8148820386326501</v>
+        <v>0.798197939227601</v>
       </c>
       <c r="F49" t="n">
-        <v>13.49316561608757</v>
+        <v>13.22009467453659</v>
       </c>
     </row>
   </sheetData>
@@ -49845,7 +49845,7 @@
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
@@ -49971,13 +49971,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.4889182873727026</v>
+        <v>0.4466137427200046</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>4.25951544396633</v>
+        <v>3.890953117807524</v>
       </c>
     </row>
     <row r="5">
@@ -50064,13 +50064,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.5978129374332963</v>
+        <v>0.5331386979515532</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>5.208218848355098</v>
+        <v>4.644769026552221</v>
       </c>
     </row>
     <row r="8">
@@ -50157,13 +50157,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.7665415945706923</v>
+        <v>0.6591729694400087</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>6.678203382536714</v>
+        <v>5.742794892509613</v>
       </c>
     </row>
     <row r="11">
@@ -50250,13 +50250,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.4719907561291904</v>
+        <v>0.4327487619672488</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>4.11204073781978</v>
+        <v>3.770159723140091</v>
       </c>
     </row>
     <row r="14">
@@ -50343,13 +50343,13 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.1751931115461214</v>
+        <v>0.1705279978753513</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>1.526303645374512</v>
+        <v>1.48566060902105</v>
       </c>
     </row>
     <row r="17">
@@ -50436,13 +50436,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.2502295076806887</v>
+        <v>0.2402167163331886</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>2.180029833266353</v>
+        <v>2.092797180117403</v>
       </c>
     </row>
     <row r="20">
@@ -50529,13 +50529,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.4466081090382062</v>
+        <v>0.411741335499582</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>3.890904036483068</v>
+        <v>3.587140474754075</v>
       </c>
     </row>
     <row r="23">
@@ -50622,13 +50622,13 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.2130306934677393</v>
+        <v>0.2059444527230841</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>1.855949250212796</v>
+        <v>1.794213061017291</v>
       </c>
     </row>
     <row r="26">
@@ -50715,13 +50715,13 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.1418411956117915</v>
+        <v>0.1388623491285609</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>1.235737706899295</v>
+        <v>1.209785634891637</v>
       </c>
     </row>
     <row r="29">
@@ -50808,13 +50808,13 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.08841310031021658</v>
+        <v>0.08730918641002414</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>0.7702656577728531</v>
+        <v>0.7606482259286403</v>
       </c>
     </row>
     <row r="32">
@@ -50901,13 +50901,13 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.08772722982162229</v>
+        <v>0.08664108610679482</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0.7642902708540547</v>
+        <v>0.7548276550209335</v>
       </c>
     </row>
     <row r="35">
@@ -50994,13 +50994,13 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.03773097278434188</v>
+        <v>0.0375400448755643</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>0.328716813098594</v>
+        <v>0.3270534259909345</v>
       </c>
     </row>
     <row r="38">
@@ -51087,13 +51087,13 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.9321475340324386</v>
+        <v>0.7770496917048596</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>8.120982421423706</v>
+        <v>6.769751199810029</v>
       </c>
     </row>
     <row r="41">
@@ -51180,10 +51180,10 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.6028304385168133</v>
+        <v>0.5339487769586027</v>
       </c>
       <c r="F43" t="n">
-        <v>2.009434808827113</v>
+        <v>1.779829268756247</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
@@ -51366,13 +51366,13 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.4888088436659583</v>
+        <v>0.4465255947933026</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
       </c>
       <c r="G49" t="n">
-        <v>4.258561957113488</v>
+        <v>3.890185162374394</v>
       </c>
     </row>
     <row r="50">
@@ -51434,7 +51434,7 @@
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>1.152119218130909e-06</v>
+        <v>1.152119218133917e-06</v>
       </c>
     </row>
     <row r="52">
@@ -51459,13 +51459,13 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.5977117828681379</v>
+        <v>0.5330931618207985</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>5.207337577509544</v>
+        <v>4.644372310255811</v>
       </c>
     </row>
     <row r="53">
@@ -51527,7 +51527,7 @@
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>1.477297138372183e-06</v>
+        <v>1.477297138374132e-06</v>
       </c>
     </row>
     <row r="55">
@@ -51552,13 +51552,13 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.7664795489360434</v>
+        <v>0.6592246849394818</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>6.677662833439157</v>
+        <v>5.743245444216068</v>
       </c>
     </row>
     <row r="56">
@@ -51620,7 +51620,7 @@
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>1.796457423788977e-06</v>
+        <v>1.796457423789815e-06</v>
       </c>
     </row>
     <row r="58">
@@ -51645,13 +51645,13 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.4719907561291894</v>
+        <v>0.4328313151592937</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>4.112040737819772</v>
+        <v>3.770878936565977</v>
       </c>
     </row>
     <row r="59">
@@ -51738,13 +51738,13 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.175130732228703</v>
+        <v>0.1704408748120532</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
       </c>
       <c r="G61" t="n">
-        <v>1.525760189192182</v>
+        <v>1.484901582322254</v>
       </c>
     </row>
     <row r="62">
@@ -51831,13 +51831,13 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.250147257063104</v>
+        <v>0.2401108988076403</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>2.17931325590583</v>
+        <v>2.091875284995133</v>
       </c>
     </row>
     <row r="65">
@@ -51924,13 +51924,13 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.4464990808599396</v>
+        <v>0.4116419777413037</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>3.889954169764746</v>
+        <v>3.586274857908075</v>
       </c>
     </row>
     <row r="68">
@@ -52017,13 +52017,13 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.2129607662239577</v>
+        <v>0.2058728012387693</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>1.855340035580139</v>
+        <v>1.793588824591866</v>
       </c>
     </row>
     <row r="71">
@@ -52110,13 +52110,13 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.1417790575484207</v>
+        <v>0.1387888528803883</v>
       </c>
       <c r="F73" t="n">
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>1.235196352551501</v>
+        <v>1.209145326659651</v>
       </c>
     </row>
     <row r="74">
@@ -52203,13 +52203,13 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.08836676918583429</v>
+        <v>0.08725056216107122</v>
       </c>
       <c r="F76" t="n">
         <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>0.769862015395508</v>
+        <v>0.760137484358401</v>
       </c>
     </row>
     <row r="77">
@@ -52296,13 +52296,13 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.0876811598980054</v>
+        <v>0.08658275004297172</v>
       </c>
       <c r="F79" t="n">
         <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>0.7638889040894715</v>
+        <v>0.7543194241545127</v>
       </c>
     </row>
     <row r="80">
@@ -52389,13 +52389,13 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>0.03770804446909932</v>
+        <v>0.0375096528061156</v>
       </c>
       <c r="F82" t="n">
         <v>0</v>
       </c>
       <c r="G82" t="n">
-        <v>0.3285170588341245</v>
+        <v>0.3267886465941787</v>
       </c>
     </row>
     <row r="83">
@@ -52457,7 +52457,7 @@
         <v>0</v>
       </c>
       <c r="G84" t="n">
-        <v>1.796456939176894e-06</v>
+        <v>1.796456939177921e-06</v>
       </c>
     </row>
     <row r="85">
@@ -52482,13 +52482,13 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0.9321475340324397</v>
+        <v>0.777217404159539</v>
       </c>
       <c r="F85" t="n">
         <v>0</v>
       </c>
       <c r="G85" t="n">
-        <v>8.120982421423713</v>
+        <v>6.771212331065084</v>
       </c>
     </row>
     <row r="86">
@@ -52550,7 +52550,7 @@
         <v>0</v>
       </c>
       <c r="G87" t="n">
-        <v>1.201574797876689e-06</v>
+        <v>1.201574797876313e-06</v>
       </c>
     </row>
     <row r="88">
@@ -52575,13 +52575,13 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>0.6027463464711875</v>
+        <v>0.5339254457793412</v>
       </c>
       <c r="F88" t="n">
-        <v>2.010000853576211</v>
+        <v>1.780933820839841</v>
       </c>
       <c r="G88" t="n">
-        <v>0.002212288549591288</v>
+        <v>0.003093256238740697</v>
       </c>
     </row>
     <row r="89">
@@ -52643,7 +52643,7 @@
         <v>0</v>
       </c>
       <c r="G90" t="n">
-        <v>1.796456701567109e-06</v>
+        <v>1.79645670156778e-06</v>
       </c>
     </row>
     <row r="91">
@@ -52668,13 +52668,13 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.0003795673478593708</v>
+        <v>0.0008067785718412335</v>
       </c>
       <c r="F91" t="n">
         <v>0</v>
       </c>
       <c r="G91" t="n">
-        <v>0.003306836789656888</v>
+        <v>0.007028752810053319</v>
       </c>
     </row>
     <row r="92">
@@ -52736,7 +52736,7 @@
         <v>0</v>
       </c>
       <c r="G93" t="n">
-        <v>1.627507187099931e-06</v>
+        <v>1.627507187099879e-06</v>
       </c>
     </row>
     <row r="94">
@@ -52761,13 +52761,13 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.09353428310680142</v>
+        <v>0.09161923871409958</v>
       </c>
       <c r="F94" t="n">
         <v>0</v>
       </c>
       <c r="G94" t="n">
-        <v>0.8148820236908642</v>
+        <v>0.7981979245749766</v>
       </c>
     </row>
   </sheetData>
@@ -55732,7 +55732,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>9.71883776301433e-06</v>
+        <v>8.880289940591441e-06</v>
       </c>
     </row>
     <row r="99">
@@ -55912,7 +55912,7 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>1.782194171617063e-05</v>
+        <v>1.782194171617062e-05</v>
       </c>
     </row>
     <row r="105">
@@ -56002,7 +56002,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>1.188412182392361e-05</v>
+        <v>1.060190479004167e-05</v>
       </c>
     </row>
     <row r="108">
@@ -56182,7 +56182,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>2.285206520578636e-05</v>
+        <v>2.285206520578635e-05</v>
       </c>
     </row>
     <row r="114">
@@ -56272,7 +56272,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1.523968005347403e-05</v>
+        <v>1.311034889493292e-05</v>
       </c>
     </row>
     <row r="117">
@@ -56542,7 +56542,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>1.853849951212403e-05</v>
+        <v>1.700455317812521e-05</v>
       </c>
     </row>
     <row r="126">
@@ -56812,7 +56812,7 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>3.482071152975758e-06</v>
+        <v>3.389647544749844e-06</v>
       </c>
     </row>
     <row r="135">
@@ -56992,7 +56992,7 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>7.459817631069128e-06</v>
+        <v>7.459817631069127e-06</v>
       </c>
     </row>
     <row r="141">
@@ -57082,7 +57082,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>4.973601930002597e-06</v>
+        <v>4.775212046455884e-06</v>
       </c>
     </row>
     <row r="144">
@@ -57262,7 +57262,7 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>1.331423756856658e-05</v>
+        <v>1.331423756856657e-05</v>
       </c>
     </row>
     <row r="150">
@@ -57352,7 +57352,7 @@
         </is>
       </c>
       <c r="F152" t="n">
-        <v>8.877605600724894e-06</v>
+        <v>8.186541055397741e-06</v>
       </c>
     </row>
     <row r="153">
@@ -57622,7 +57622,7 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>8.364513144222424e-06</v>
+        <v>8.088081238393072e-06</v>
       </c>
     </row>
     <row r="162">
@@ -57802,7 +57802,7 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>8.351091877222378e-06</v>
+        <v>8.35109187722238e-06</v>
       </c>
     </row>
     <row r="168">
@@ -57892,7 +57892,7 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>5.568691192751039e-06</v>
+        <v>5.452568118202464e-06</v>
       </c>
     </row>
     <row r="171">
@@ -58072,7 +58072,7 @@
         </is>
       </c>
       <c r="F176" t="n">
-        <v>5.205440139560555e-06</v>
+        <v>5.205440139560551e-06</v>
       </c>
     </row>
     <row r="177">
@@ -58162,7 +58162,7 @@
         </is>
       </c>
       <c r="F179" t="n">
-        <v>3.470803253158976e-06</v>
+        <v>3.427794017344996e-06</v>
       </c>
     </row>
     <row r="180">
@@ -58342,7 +58342,7 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>5.165058584029695e-06</v>
+        <v>5.165058584029697e-06</v>
       </c>
     </row>
     <row r="186">
@@ -58432,7 +58432,7 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>3.443874404016653e-06</v>
+        <v>3.401557821666196e-06</v>
       </c>
     </row>
     <row r="189">
@@ -58702,7 +58702,7 @@
         </is>
       </c>
       <c r="F197" t="n">
-        <v>1.481067916458701e-06</v>
+        <v>1.473633451762487e-06</v>
       </c>
     </row>
     <row r="198">
@@ -58882,7 +58882,7 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>2.778909540077649e-05</v>
+        <v>2.77890954007765e-05</v>
       </c>
     </row>
     <row r="204">
@@ -58972,7 +58972,7 @@
         </is>
       </c>
       <c r="F206" t="n">
-        <v>1.853360627952582e-05</v>
+        <v>1.545693231539271e-05</v>
       </c>
     </row>
     <row r="207">
@@ -59152,7 +59152,7 @@
         </is>
       </c>
       <c r="F212" t="n">
-        <v>1.8586961903277e-05</v>
+        <v>1.858696190327699e-05</v>
       </c>
     </row>
     <row r="213">
@@ -59242,7 +59242,7 @@
         </is>
       </c>
       <c r="F215" t="n">
-        <v>1.239479717596365e-05</v>
+        <v>1.098224085521036e-05</v>
       </c>
     </row>
     <row r="216">
@@ -59422,7 +59422,7 @@
         </is>
       </c>
       <c r="F221" t="n">
-        <v>2.778909172521557e-05</v>
+        <v>2.778909172521556e-05</v>
       </c>
     </row>
     <row r="222">
@@ -59512,7 +59512,7 @@
         </is>
       </c>
       <c r="F224" t="n">
-        <v>1.852722661762873e-05</v>
+        <v>8.098786101500827e-06</v>
       </c>
     </row>
     <row r="225">
@@ -59782,7 +59782,7 @@
         </is>
       </c>
       <c r="F233" t="n">
-        <v>1.774141286731019e-05</v>
+        <v>1.738236707674677e-05</v>
       </c>
     </row>
     <row r="234">
@@ -62862,7 +62862,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>9.71883776301433e-06</v>
+        <v>8.880289940591441e-06</v>
       </c>
     </row>
     <row r="9">
@@ -63042,7 +63042,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.782194171617063e-05</v>
+        <v>1.782194171617062e-05</v>
       </c>
     </row>
     <row r="15">
@@ -63132,7 +63132,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1.188412182392361e-05</v>
+        <v>1.060190479004167e-05</v>
       </c>
     </row>
     <row r="18">
@@ -63312,7 +63312,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.285206520578636e-05</v>
+        <v>2.285206520578635e-05</v>
       </c>
     </row>
     <row r="24">
@@ -63402,7 +63402,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1.523968005347403e-05</v>
+        <v>1.311034889493292e-05</v>
       </c>
     </row>
     <row r="27">
@@ -63672,7 +63672,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1.853849951212403e-05</v>
+        <v>1.700455317812521e-05</v>
       </c>
     </row>
     <row r="36">
@@ -63942,7 +63942,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.482071152975758e-06</v>
+        <v>3.389647544749844e-06</v>
       </c>
     </row>
     <row r="45">
@@ -64122,7 +64122,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>7.459817631069128e-06</v>
+        <v>7.459817631069127e-06</v>
       </c>
     </row>
     <row r="51">
@@ -64212,7 +64212,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>4.973601930002597e-06</v>
+        <v>4.775212046455884e-06</v>
       </c>
     </row>
     <row r="54">
@@ -64392,7 +64392,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>1.331423756856658e-05</v>
+        <v>1.331423756856657e-05</v>
       </c>
     </row>
     <row r="60">
@@ -64482,7 +64482,7 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>8.877605600724894e-06</v>
+        <v>8.186541055397741e-06</v>
       </c>
     </row>
     <row r="63">
@@ -64752,7 +64752,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>8.364513144222424e-06</v>
+        <v>8.088081238393072e-06</v>
       </c>
     </row>
     <row r="72">
@@ -64932,7 +64932,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>8.351091877222378e-06</v>
+        <v>8.35109187722238e-06</v>
       </c>
     </row>
     <row r="78">
@@ -65022,7 +65022,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>5.568691192751039e-06</v>
+        <v>5.452568118202464e-06</v>
       </c>
     </row>
     <row r="81">
@@ -65202,7 +65202,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>5.205440139560555e-06</v>
+        <v>5.205440139560551e-06</v>
       </c>
     </row>
     <row r="87">
@@ -65292,7 +65292,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>3.470803253158976e-06</v>
+        <v>3.427794017344996e-06</v>
       </c>
     </row>
     <row r="90">
@@ -65472,7 +65472,7 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>5.165058584029695e-06</v>
+        <v>5.165058584029697e-06</v>
       </c>
     </row>
     <row r="96">
@@ -65562,7 +65562,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>3.443874404016653e-06</v>
+        <v>3.401557821666196e-06</v>
       </c>
     </row>
     <row r="99">
@@ -65832,7 +65832,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>1.481067916458701e-06</v>
+        <v>1.473633451762487e-06</v>
       </c>
     </row>
     <row r="108">
@@ -66012,7 +66012,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>2.778909540077649e-05</v>
+        <v>2.77890954007765e-05</v>
       </c>
     </row>
     <row r="114">
@@ -66102,7 +66102,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>1.853360627952582e-05</v>
+        <v>1.545693231539271e-05</v>
       </c>
     </row>
     <row r="117">
@@ -66282,7 +66282,7 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>1.8586961903277e-05</v>
+        <v>1.858696190327699e-05</v>
       </c>
     </row>
     <row r="123">
@@ -66372,7 +66372,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>1.239479717596365e-05</v>
+        <v>1.098224085521036e-05</v>
       </c>
     </row>
     <row r="126">
@@ -66552,7 +66552,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>2.778909172521557e-05</v>
+        <v>2.778909172521556e-05</v>
       </c>
     </row>
     <row r="132">
@@ -66642,7 +66642,7 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>1.852722661762873e-05</v>
+        <v>8.098786101500827e-06</v>
       </c>
     </row>
     <row r="135">
@@ -66912,7 +66912,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>1.774141286731019e-05</v>
+        <v>1.738236707674677e-05</v>
       </c>
     </row>
     <row r="144">

</xml_diff>